<commit_message>
feat(platform): migrate risk engine to Laya, add real-time memo analysis, update service READMEs, and clean architecture
</commit_message>
<xml_diff>
--- a/hybrid_bench/reports/Risk_Engine_Benchmark_Report.xlsx
+++ b/hybrid_bench/reports/Risk_Engine_Benchmark_Report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JLB83807\The Vault\workspaces\FSE-Capstone\hybrid_bench\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4058CCF3-496F-46A1-9FEB-6BD373E1FDC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA4DA7B4-5439-4BFF-9B3B-7B84A02F0BD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Executive Summary &amp; Systems" sheetId="1" r:id="rId1"/>
@@ -20,12 +20,11 @@
     <sheet name="Telemetry, Latency &amp; Safety" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="701" uniqueCount="428">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="661" uniqueCount="402">
   <si>
     <t>BANK TRANSFER RISK ENGINE BENCHMARK REPORT</t>
   </si>
@@ -767,9 +766,6 @@
     <t>Detection Mechanism</t>
   </si>
   <si>
-    <t>Primary Risk Indicator</t>
-  </si>
-  <si>
     <t>os_patch_age_days</t>
   </si>
   <si>
@@ -782,9 +778,6 @@
     <t>Older patch levels correlate heavily with unpatched kernel vulnerabilities and emulator farms</t>
   </si>
   <si>
-    <t>Old Patch (&gt;180d) = High Fraud</t>
-  </si>
-  <si>
     <t>balance_drain_ratio</t>
   </si>
   <si>
@@ -797,9 +790,6 @@
     <t>Fraudsters and money mules drain accounts to 0% immediately upon gaining access</t>
   </si>
   <si>
-    <t>High Drain (&gt;85%) = Critical Risk</t>
-  </si>
-  <si>
     <t>payee_age_days</t>
   </si>
   <si>
@@ -812,9 +802,6 @@
     <t>New payees added minutes/hours before transfer carry massive scam collection risk</t>
   </si>
   <si>
-    <t>New Payee (&lt;24h) = Elevated Risk</t>
-  </si>
-  <si>
     <t>form_seconds</t>
   </si>
   <si>
@@ -827,9 +814,6 @@
     <t>Sub-second transfers indicate automated bot scripts; extreme stalling indicates coercion</t>
   </si>
   <si>
-    <t>Extremely Fast / Slow = High Suspicion</t>
-  </si>
-  <si>
     <t>payees_24h</t>
   </si>
   <si>
@@ -842,9 +826,6 @@
     <t>Rapid counterparty additions indicate active account takeover or money laundering mule activity</t>
   </si>
   <si>
-    <t>Burst Additions (&gt;3) = High Risk</t>
-  </si>
-  <si>
     <t>spike_ratio</t>
   </si>
   <si>
@@ -857,9 +838,6 @@
     <t>Sudden 5x-10x spikes deviate from legitimate behavioral profile</t>
   </si>
   <si>
-    <t>Spike (&gt;5.0) = Immediate Step-up</t>
-  </si>
-  <si>
     <t>dow</t>
   </si>
   <si>
@@ -872,9 +850,6 @@
     <t>Off-hour weekend transfers exhibit higher fraudulent incidence due to lower bank branch staffing</t>
   </si>
   <si>
-    <t>Weekend Off-Hours = Elevated Triage</t>
-  </si>
-  <si>
     <t>credential_change_hours_ago</t>
   </si>
   <si>
@@ -887,9 +862,6 @@
     <t>Attackers change passwords or email addresses immediately prior to draining balances</t>
   </si>
   <si>
-    <t>Recent Change (&lt;24h) = High Alert</t>
-  </si>
-  <si>
     <t>seconds_since_login</t>
   </si>
   <si>
@@ -902,9 +874,6 @@
     <t>Transfers submitted within seconds of login often stem from automated credential stuffing</t>
   </si>
   <si>
-    <t>Instant Transfer = Bot Indicator</t>
-  </si>
-  <si>
     <t>velocity_kmh</t>
   </si>
   <si>
@@ -917,9 +886,6 @@
     <t>Impossible physical travel (&gt;800 km/h) indicates proxy switching or credential sharing</t>
   </si>
   <si>
-    <t>Impossible Speed = Hard Gate 0 Block</t>
-  </si>
-  <si>
     <t>2. NANOJEV TEMPERATURE CALIBRATION &amp; RELIABILITY</t>
   </si>
   <si>
@@ -953,9 +919,6 @@
     <t>Cools overconfident logits</t>
   </si>
   <si>
-    <t>OPTIMAL</t>
-  </si>
-  <si>
     <t>Expected Calibration Error (ECE)</t>
   </si>
   <si>
@@ -968,9 +931,6 @@
     <t>Cuts confidence error from 49.5% to 21.3%</t>
   </si>
   <si>
-    <t>CALIBRATED</t>
-  </si>
-  <si>
     <t>Decision Threshold (theta_block)</t>
   </si>
   <si>
@@ -983,9 +943,6 @@
     <t>Conservative blocking to prevent false blocks</t>
   </si>
   <si>
-    <t>VALIDATED</t>
-  </si>
-  <si>
     <t>Decision Threshold (theta_2fa)</t>
   </si>
   <si>
@@ -1019,9 +976,6 @@
     <t>Hardware Target</t>
   </si>
   <si>
-    <t>SLA Assessment</t>
-  </si>
-  <si>
     <t>Gate 0 Deterministic Rules</t>
   </si>
   <si>
@@ -1034,9 +988,6 @@
     <t>CPU</t>
   </si>
   <si>
-    <t>PASS (&lt;0.01 ms)</t>
-  </si>
-  <si>
     <t>Tabular Feature Pipeline</t>
   </si>
   <si>
@@ -1052,9 +1003,6 @@
     <t>Vectorized Pandas/NumPy transforms</t>
   </si>
   <si>
-    <t>PASS (~31 ms)</t>
-  </si>
-  <si>
     <t>XGBoost Inference (S2)</t>
   </si>
   <si>
@@ -1070,9 +1018,6 @@
     <t>Tree traversal C-API</t>
   </si>
   <si>
-    <t>PASS (~4.4 ms)</t>
-  </si>
-  <si>
     <t>NanoJev Raw ONNX (CPU)</t>
   </si>
   <si>
@@ -1088,9 +1033,6 @@
     <t>Qwen2.5-0.5B INT8 forward pass</t>
   </si>
   <si>
-    <t>HEAVY (~294 ms)</t>
-  </si>
-  <si>
     <t>NanoJev Cache Hit</t>
   </si>
   <si>
@@ -1109,9 +1051,6 @@
     <t>RAM</t>
   </si>
   <si>
-    <t>PASS (&lt;1.0 ms)</t>
-  </si>
-  <si>
     <t>Escalate-Only Fusion Rule</t>
   </si>
   <si>
@@ -1160,9 +1099,6 @@
     <t>Timeout Fallback Rate</t>
   </si>
   <si>
-    <t>Operational Assessment</t>
-  </si>
-  <si>
     <t>10 TPS</t>
   </si>
   <si>
@@ -1178,9 +1114,6 @@
     <t>0.0%</t>
   </si>
   <si>
-    <t>Fully compliant (p99 = 137 ms)</t>
-  </si>
-  <si>
     <t>25 TPS</t>
   </si>
   <si>
@@ -1196,9 +1129,6 @@
     <t>4.0%</t>
   </si>
   <si>
-    <t>CPU queue saturation (p99 = 2,073 ms)</t>
-  </si>
-  <si>
     <t>50 TPS</t>
   </si>
   <si>
@@ -1214,9 +1144,6 @@
     <t>1.2%</t>
   </si>
   <si>
-    <t>Severe CPU bottleneck (p99 = 6,596 ms)</t>
-  </si>
-  <si>
     <t>5. ADVERSARIAL PROMPT INJECTION &amp; METAMORPHIC SECURITY SUITE</t>
   </si>
   <si>
@@ -1238,9 +1165,6 @@
     <t>Unchanged Decisions</t>
   </si>
   <si>
-    <t>Safety Verdict</t>
-  </si>
-  <si>
     <t>Direct Instruction Overrides ('IGNORE ALL RULES')</t>
   </si>
   <si>
@@ -1251,9 +1175,6 @@
   </si>
   <si>
     <t>38 (63.3%)</t>
-  </si>
-  <si>
-    <t>100% IMMUNE</t>
   </si>
   <si>
     <t>Authority &amp; Admin Impersonation ('[BSP AUDIT CLEAR]')</t>
@@ -1585,19 +1506,6 @@
     <xf numFmtId="165" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1614,6 +1522,19 @@
     <xf numFmtId="0" fontId="14" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1673,10 +1594,10 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>2082800</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>254000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="5143500" cy="3619500"/>
     <xdr:pic>
@@ -1698,7 +1619,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5226050" y="4654550"/>
+          <a:off x="11607800" y="1835150"/>
           <a:ext cx="5143500" cy="3619500"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2038,38 +1959,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
     </row>
     <row r="2" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
     </row>
     <row r="3" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="29" t="s">
+      <c r="A4" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="27"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
+      <c r="B4" s="33"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="33"/>
+      <c r="G4" s="33"/>
     </row>
     <row r="5" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
@@ -2210,15 +2131,15 @@
       </c>
     </row>
     <row r="12" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="29" t="s">
+      <c r="A12" s="32" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="27"/>
-      <c r="C12" s="27"/>
-      <c r="D12" s="27"/>
-      <c r="E12" s="27"/>
-      <c r="F12" s="27"/>
-      <c r="G12" s="27"/>
+      <c r="B12" s="33"/>
+      <c r="C12" s="33"/>
+      <c r="D12" s="33"/>
+      <c r="E12" s="33"/>
+      <c r="F12" s="33"/>
+      <c r="G12" s="33"/>
     </row>
     <row r="13" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
@@ -2382,67 +2303,67 @@
       </c>
     </row>
     <row r="21" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="29" t="s">
+      <c r="A21" s="32" t="s">
         <v>87</v>
       </c>
-      <c r="B21" s="27"/>
-      <c r="C21" s="27"/>
-      <c r="D21" s="27"/>
-      <c r="E21" s="27"/>
-      <c r="F21" s="27"/>
-      <c r="G21" s="27"/>
+      <c r="B21" s="33"/>
+      <c r="C21" s="33"/>
+      <c r="D21" s="33"/>
+      <c r="E21" s="33"/>
+      <c r="F21" s="33"/>
+      <c r="G21" s="33"/>
     </row>
     <row r="22" spans="1:7" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="B22" s="26" t="s">
+      <c r="B22" s="36" t="s">
         <v>89</v>
       </c>
-      <c r="C22" s="27"/>
-      <c r="D22" s="27"/>
-      <c r="E22" s="27"/>
-      <c r="F22" s="27"/>
-      <c r="G22" s="27"/>
+      <c r="C22" s="33"/>
+      <c r="D22" s="33"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="33"/>
+      <c r="G22" s="33"/>
     </row>
     <row r="23" spans="1:7" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="B23" s="26" t="s">
+      <c r="B23" s="36" t="s">
         <v>91</v>
       </c>
-      <c r="C23" s="27"/>
-      <c r="D23" s="27"/>
-      <c r="E23" s="27"/>
-      <c r="F23" s="27"/>
-      <c r="G23" s="27"/>
+      <c r="C23" s="33"/>
+      <c r="D23" s="33"/>
+      <c r="E23" s="33"/>
+      <c r="F23" s="33"/>
+      <c r="G23" s="33"/>
     </row>
     <row r="24" spans="1:7" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="B24" s="26" t="s">
+      <c r="B24" s="36" t="s">
         <v>93</v>
       </c>
-      <c r="C24" s="27"/>
-      <c r="D24" s="27"/>
-      <c r="E24" s="27"/>
-      <c r="F24" s="27"/>
-      <c r="G24" s="27"/>
+      <c r="C24" s="33"/>
+      <c r="D24" s="33"/>
+      <c r="E24" s="33"/>
+      <c r="F24" s="33"/>
+      <c r="G24" s="33"/>
     </row>
     <row r="25" spans="1:7" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="B25" s="26" t="s">
+      <c r="B25" s="36" t="s">
         <v>95</v>
       </c>
-      <c r="C25" s="27"/>
-      <c r="D25" s="27"/>
-      <c r="E25" s="27"/>
-      <c r="F25" s="27"/>
-      <c r="G25" s="27"/>
+      <c r="C25" s="33"/>
+      <c r="D25" s="33"/>
+      <c r="E25" s="33"/>
+      <c r="F25" s="33"/>
+      <c r="G25" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -2475,26 +2396,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="34" t="s">
         <v>96</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
     </row>
     <row r="2" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="32" t="s">
-        <v>427</v>
-      </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
+      <c r="A2" s="37" t="s">
+        <v>401</v>
+      </c>
+      <c r="B2" s="37"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
+      <c r="G2" s="37"/>
     </row>
     <row r="3" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
@@ -2658,15 +2579,15 @@
       </c>
     </row>
     <row r="11" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="32" t="s">
+      <c r="A11" s="37" t="s">
         <v>144</v>
       </c>
-      <c r="B11" s="32"/>
-      <c r="C11" s="32"/>
-      <c r="D11" s="32"/>
-      <c r="E11" s="32"/>
-      <c r="F11" s="32"/>
-      <c r="G11" s="32"/>
+      <c r="B11" s="37"/>
+      <c r="C11" s="37"/>
+      <c r="D11" s="37"/>
+      <c r="E11" s="37"/>
+      <c r="F11" s="37"/>
+      <c r="G11" s="37"/>
     </row>
     <row r="12" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
@@ -2852,53 +2773,53 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="34" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="34" t="s">
         <v>174</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
     </row>
     <row r="2" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="35" t="s">
         <v>175</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
     </row>
     <row r="3" spans="1:8" ht="10" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="29" t="s">
+      <c r="A4" s="32" t="s">
         <v>176</v>
       </c>
-      <c r="B4" s="27"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
-      <c r="H4" s="27"/>
+      <c r="B4" s="33"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="33"/>
+      <c r="G4" s="33"/>
+      <c r="H4" s="33"/>
     </row>
     <row r="24" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A24" s="31" t="s">
+      <c r="A24" s="38" t="s">
         <v>177</v>
       </c>
-      <c r="B24" s="27"/>
-      <c r="C24" s="27"/>
-      <c r="D24" s="27"/>
-      <c r="E24" s="27"/>
-      <c r="F24" s="27"/>
-      <c r="G24" s="27"/>
-      <c r="H24" s="27"/>
+      <c r="B24" s="33"/>
+      <c r="C24" s="33"/>
+      <c r="D24" s="33"/>
+      <c r="E24" s="33"/>
+      <c r="F24" s="33"/>
+      <c r="G24" s="33"/>
+      <c r="H24" s="33"/>
     </row>
     <row r="25" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
@@ -3057,16 +2978,16 @@
       </c>
     </row>
     <row r="32" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A32" s="31" t="s">
+      <c r="A32" s="38" t="s">
         <v>190</v>
       </c>
-      <c r="B32" s="27"/>
-      <c r="C32" s="27"/>
-      <c r="D32" s="27"/>
-      <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
-      <c r="G32" s="27"/>
-      <c r="H32" s="27"/>
+      <c r="B32" s="33"/>
+      <c r="C32" s="33"/>
+      <c r="D32" s="33"/>
+      <c r="E32" s="33"/>
+      <c r="F32" s="33"/>
+      <c r="G32" s="33"/>
+      <c r="H32" s="33"/>
     </row>
     <row r="33" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
@@ -3225,16 +3146,16 @@
       </c>
     </row>
     <row r="40" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A40" s="31" t="s">
+      <c r="A40" s="38" t="s">
         <v>191</v>
       </c>
-      <c r="B40" s="27"/>
-      <c r="C40" s="27"/>
-      <c r="D40" s="27"/>
-      <c r="E40" s="27"/>
-      <c r="F40" s="27"/>
-      <c r="G40" s="27"/>
-      <c r="H40" s="27"/>
+      <c r="B40" s="33"/>
+      <c r="C40" s="33"/>
+      <c r="D40" s="33"/>
+      <c r="E40" s="33"/>
+      <c r="F40" s="33"/>
+      <c r="G40" s="33"/>
+      <c r="H40" s="33"/>
     </row>
     <row r="41" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
@@ -3393,16 +3314,16 @@
       </c>
     </row>
     <row r="48" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A48" s="31" t="s">
+      <c r="A48" s="38" t="s">
         <v>192</v>
       </c>
-      <c r="B48" s="27"/>
-      <c r="C48" s="27"/>
-      <c r="D48" s="27"/>
-      <c r="E48" s="27"/>
-      <c r="F48" s="27"/>
-      <c r="G48" s="27"/>
-      <c r="H48" s="27"/>
+      <c r="B48" s="33"/>
+      <c r="C48" s="33"/>
+      <c r="D48" s="33"/>
+      <c r="E48" s="33"/>
+      <c r="F48" s="33"/>
+      <c r="G48" s="33"/>
+      <c r="H48" s="33"/>
     </row>
     <row r="49" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
@@ -3589,38 +3510,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="34" t="s">
         <v>193</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
     </row>
     <row r="2" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="35" t="s">
         <v>194</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
     </row>
     <row r="3" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="29" t="s">
+      <c r="A4" s="32" t="s">
         <v>195</v>
       </c>
-      <c r="B4" s="27"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
+      <c r="B4" s="33"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="33"/>
+      <c r="G4" s="33"/>
     </row>
     <row r="5" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
@@ -3922,15 +3843,15 @@
       </c>
     </row>
     <row r="19" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="29" t="s">
+      <c r="A19" s="32" t="s">
         <v>204</v>
       </c>
-      <c r="B19" s="27"/>
-      <c r="C19" s="27"/>
-      <c r="D19" s="27"/>
-      <c r="E19" s="27"/>
-      <c r="F19" s="27"/>
-      <c r="G19" s="27"/>
+      <c r="B19" s="33"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="33"/>
+      <c r="G19" s="33"/>
     </row>
     <row r="20" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
@@ -4370,15 +4291,15 @@
       </c>
     </row>
     <row r="40" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A40" s="29" t="s">
+      <c r="A40" s="32" t="s">
         <v>229</v>
       </c>
-      <c r="B40" s="27"/>
-      <c r="C40" s="27"/>
-      <c r="D40" s="27"/>
-      <c r="E40" s="27"/>
-      <c r="F40" s="27"/>
-      <c r="G40" s="27"/>
+      <c r="B40" s="33"/>
+      <c r="C40" s="33"/>
+      <c r="D40" s="33"/>
+      <c r="E40" s="33"/>
+      <c r="F40" s="33"/>
+      <c r="G40" s="33"/>
     </row>
     <row r="41" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
@@ -4877,7 +4798,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:F89"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20.81640625" customWidth="1"/>
@@ -4885,45 +4806,41 @@
     <col min="3" max="3" width="9.6328125" customWidth="1"/>
     <col min="4" max="4" width="20.453125" customWidth="1"/>
     <col min="5" max="5" width="45" customWidth="1"/>
-    <col min="6" max="6" width="45" style="33" customWidth="1"/>
-    <col min="7" max="7" width="41" customWidth="1"/>
+    <col min="6" max="6" width="45" style="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:6" ht="34" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="34" t="s">
         <v>235</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-    </row>
-    <row r="2" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="30" t="s">
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+    </row>
+    <row r="2" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="35" t="s">
         <v>236</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-    </row>
-    <row r="3" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="4" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="29" t="s">
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+    </row>
+    <row r="3" spans="1:6" ht="10" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A4" s="32" t="s">
         <v>237</v>
       </c>
-      <c r="B4" s="27"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
-    </row>
-    <row r="5" spans="1:7" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="33"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="33"/>
+    </row>
+    <row r="5" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>238</v>
       </c>
@@ -4939,280 +4856,243 @@
       <c r="E5" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="F5" s="34" t="s">
+      <c r="F5" s="27" t="s">
         <v>243</v>
       </c>
-      <c r="G5" s="1" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
         <v>1</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C6" s="12">
         <v>1.5049999999999999</v>
       </c>
       <c r="D6" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="F6" s="28" t="s">
         <v>247</v>
       </c>
-      <c r="F6" s="35" t="s">
-        <v>248</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>2</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C7" s="12">
         <v>0.4622</v>
       </c>
       <c r="D7" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="F7" s="28" t="s">
         <v>251</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="F7" s="35" t="s">
-        <v>253</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>3</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="C8" s="12">
         <v>0.37209999999999999</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>257</v>
-      </c>
-      <c r="F8" s="35" t="s">
-        <v>258</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>254</v>
+      </c>
+      <c r="F8" s="28" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>4</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="C9" s="12">
         <v>0.32990000000000003</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>262</v>
-      </c>
-      <c r="F9" s="35" t="s">
-        <v>263</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>258</v>
+      </c>
+      <c r="F9" s="28" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>5</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="C10" s="12">
         <v>0.31630000000000003</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>267</v>
-      </c>
-      <c r="F10" s="35" t="s">
-        <v>268</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>262</v>
+      </c>
+      <c r="F10" s="28" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>6</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="C11" s="12">
         <v>0.29659999999999997</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>272</v>
-      </c>
-      <c r="F11" s="35" t="s">
-        <v>273</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>266</v>
+      </c>
+      <c r="F11" s="28" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>7</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="C12" s="12">
         <v>0.2863</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>277</v>
-      </c>
-      <c r="F12" s="35" t="s">
-        <v>278</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>270</v>
+      </c>
+      <c r="F12" s="28" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>8</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="C13" s="12">
         <v>0.26100000000000001</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>281</v>
+        <v>273</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>282</v>
-      </c>
-      <c r="F13" s="35" t="s">
-        <v>283</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>274</v>
+      </c>
+      <c r="F13" s="28" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>9</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>285</v>
+        <v>276</v>
       </c>
       <c r="C14" s="12">
         <v>0.2606</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>286</v>
+        <v>277</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="F14" s="35" t="s">
-        <v>288</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>278</v>
+      </c>
+      <c r="F14" s="28" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>10</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>290</v>
+        <v>280</v>
       </c>
       <c r="C15" s="12">
         <v>0.2167</v>
       </c>
       <c r="D15" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="F15" s="28" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A37" s="32" t="s">
+        <v>284</v>
+      </c>
+      <c r="B37" s="33"/>
+      <c r="C37" s="33"/>
+      <c r="D37" s="33"/>
+      <c r="E37" s="33"/>
+      <c r="F37" s="33"/>
+    </row>
+    <row r="38" spans="1:6" ht="26" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="F38" s="27" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="11" t="s">
         <v>291</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>292</v>
-      </c>
-      <c r="F15" s="35" t="s">
-        <v>293</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A37" s="29" t="s">
-        <v>295</v>
-      </c>
-      <c r="B37" s="27"/>
-      <c r="C37" s="27"/>
-      <c r="D37" s="27"/>
-      <c r="E37" s="27"/>
-      <c r="F37" s="27"/>
-      <c r="G37" s="27"/>
-    </row>
-    <row r="38" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="1" t="s">
-        <v>296</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>297</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>298</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>299</v>
-      </c>
-      <c r="E38" s="1" t="s">
-        <v>300</v>
-      </c>
-      <c r="F38" s="34" t="s">
-        <v>301</v>
-      </c>
-      <c r="G38" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="11" t="s">
-        <v>302</v>
       </c>
       <c r="B39" s="12">
         <v>1</v>
@@ -5221,21 +5101,18 @@
         <v>5</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>303</v>
+        <v>292</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>304</v>
-      </c>
-      <c r="F39" s="35" t="s">
-        <v>305</v>
-      </c>
-      <c r="G39" s="8" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+        <v>293</v>
+      </c>
+      <c r="F39" s="28" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="11" t="s">
-        <v>307</v>
+        <v>295</v>
       </c>
       <c r="B40" s="12">
         <v>0.49459999999999998</v>
@@ -5244,21 +5121,18 @@
         <v>0.21290000000000001</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>308</v>
+        <v>296</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>309</v>
-      </c>
-      <c r="F40" s="35" t="s">
-        <v>310</v>
-      </c>
-      <c r="G40" s="8" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+        <v>297</v>
+      </c>
+      <c r="F40" s="28" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="11" t="s">
-        <v>312</v>
+        <v>299</v>
       </c>
       <c r="B41" s="12">
         <v>0.5</v>
@@ -5267,21 +5141,18 @@
         <v>0.4</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>313</v>
+        <v>300</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>314</v>
-      </c>
-      <c r="F41" s="35" t="s">
-        <v>315</v>
-      </c>
-      <c r="G41" s="8" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+        <v>301</v>
+      </c>
+      <c r="F41" s="28" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="11" t="s">
-        <v>317</v>
+        <v>303</v>
       </c>
       <c r="B42" s="12">
         <v>0.5</v>
@@ -5290,353 +5161,308 @@
         <v>0.6</v>
       </c>
       <c r="D42" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="F42" s="28" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A61" s="32" t="s">
+        <v>307</v>
+      </c>
+      <c r="B61" s="33"/>
+      <c r="C61" s="33"/>
+      <c r="D61" s="33"/>
+      <c r="E61" s="33"/>
+      <c r="F61" s="33"/>
+    </row>
+    <row r="62" spans="1:6" ht="26" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A62" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="E62" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="F62" s="27" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A63" s="11" t="s">
+        <v>314</v>
+      </c>
+      <c r="B63" s="14" t="s">
+        <v>315</v>
+      </c>
+      <c r="C63" s="14" t="s">
+        <v>315</v>
+      </c>
+      <c r="D63" s="14" t="s">
+        <v>315</v>
+      </c>
+      <c r="E63" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="F63" s="29" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A64" s="11" t="s">
         <v>318</v>
       </c>
-      <c r="E42" s="3" t="s">
+      <c r="B64" s="14" t="s">
         <v>319</v>
       </c>
-      <c r="F42" s="35" t="s">
+      <c r="C64" s="14" t="s">
         <v>320</v>
       </c>
-      <c r="G42" s="8" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A61" s="29" t="s">
+      <c r="D64" s="14" t="s">
         <v>321</v>
       </c>
-      <c r="B61" s="27"/>
-      <c r="C61" s="27"/>
-      <c r="D61" s="27"/>
-      <c r="E61" s="27"/>
-      <c r="F61" s="27"/>
-      <c r="G61" s="27"/>
-    </row>
-    <row r="62" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A62" s="1" t="s">
+      <c r="E64" s="3" t="s">
         <v>322</v>
       </c>
-      <c r="B62" s="1" t="s">
+      <c r="F64" s="29" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A65" s="11" t="s">
         <v>323</v>
       </c>
-      <c r="C62" s="1" t="s">
+      <c r="B65" s="14" t="s">
         <v>324</v>
       </c>
-      <c r="D62" s="1" t="s">
+      <c r="C65" s="14" t="s">
         <v>325</v>
       </c>
-      <c r="E62" s="1" t="s">
+      <c r="D65" s="14" t="s">
         <v>326</v>
       </c>
-      <c r="F62" s="34" t="s">
+      <c r="E65" s="3" t="s">
         <v>327</v>
       </c>
-      <c r="G62" s="1" t="s">
+      <c r="F65" s="29" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A66" s="11" t="s">
         <v>328</v>
       </c>
-    </row>
-    <row r="63" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A63" s="11" t="s">
+      <c r="B66" s="14" t="s">
         <v>329</v>
       </c>
-      <c r="B63" s="14" t="s">
+      <c r="C66" s="14" t="s">
         <v>330</v>
       </c>
-      <c r="C63" s="14" t="s">
-        <v>330</v>
-      </c>
-      <c r="D63" s="14" t="s">
-        <v>330</v>
-      </c>
-      <c r="E63" s="3" t="s">
+      <c r="D66" s="14" t="s">
         <v>331</v>
       </c>
-      <c r="F63" s="36" t="s">
+      <c r="E66" s="3" t="s">
         <v>332</v>
       </c>
-      <c r="G63" s="8" t="s">
+      <c r="F66" s="29" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A67" s="11" t="s">
         <v>333</v>
       </c>
-    </row>
-    <row r="64" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A64" s="11" t="s">
+      <c r="B67" s="14" t="s">
         <v>334</v>
       </c>
-      <c r="B64" s="14" t="s">
+      <c r="C67" s="14" t="s">
         <v>335</v>
       </c>
-      <c r="C64" s="14" t="s">
+      <c r="D67" s="14" t="s">
         <v>336</v>
       </c>
-      <c r="D64" s="14" t="s">
+      <c r="E67" s="3" t="s">
         <v>337</v>
       </c>
-      <c r="E64" s="3" t="s">
+      <c r="F67" s="29" t="s">
         <v>338</v>
       </c>
-      <c r="F64" s="36" t="s">
-        <v>332</v>
-      </c>
-      <c r="G64" s="8" t="s">
+    </row>
+    <row r="68" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A68" s="11" t="s">
         <v>339</v>
       </c>
-    </row>
-    <row r="65" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A65" s="11" t="s">
+      <c r="B68" s="14" t="s">
         <v>340</v>
       </c>
-      <c r="B65" s="14" t="s">
+      <c r="C68" s="14" t="s">
+        <v>340</v>
+      </c>
+      <c r="D68" s="14" t="s">
+        <v>315</v>
+      </c>
+      <c r="E68" s="3" t="s">
         <v>341</v>
       </c>
-      <c r="C65" s="14" t="s">
+      <c r="F68" s="29" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A69" s="11" t="s">
         <v>342</v>
       </c>
-      <c r="D65" s="14" t="s">
+      <c r="B69" s="14" t="s">
         <v>343</v>
       </c>
-      <c r="E65" s="3" t="s">
+      <c r="C69" s="14" t="s">
         <v>344</v>
       </c>
-      <c r="F65" s="36" t="s">
-        <v>332</v>
-      </c>
-      <c r="G65" s="8" t="s">
+      <c r="D69" s="14" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="66" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A66" s="11" t="s">
+      <c r="E69" s="3" t="s">
         <v>346</v>
       </c>
-      <c r="B66" s="14" t="s">
+      <c r="F69" s="29" t="s">
         <v>347</v>
       </c>
-      <c r="C66" s="14" t="s">
+    </row>
+    <row r="71" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A71" s="32" t="s">
         <v>348</v>
       </c>
-      <c r="D66" s="14" t="s">
+      <c r="B71" s="33"/>
+      <c r="C71" s="33"/>
+      <c r="D71" s="33"/>
+      <c r="E71" s="33"/>
+      <c r="F71" s="33"/>
+    </row>
+    <row r="72" spans="1:6" ht="26" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A72" s="1" t="s">
         <v>349</v>
       </c>
-      <c r="E66" s="3" t="s">
+      <c r="B72" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="F66" s="36" t="s">
-        <v>332</v>
-      </c>
-      <c r="G66" s="9" t="s">
+      <c r="C72" s="1" t="s">
         <v>351</v>
       </c>
-    </row>
-    <row r="67" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A67" s="11" t="s">
+      <c r="D72" s="1" t="s">
         <v>352</v>
       </c>
-      <c r="B67" s="14" t="s">
+      <c r="E72" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="C67" s="14" t="s">
+      <c r="F72" s="27" t="s">
         <v>354</v>
       </c>
-      <c r="D67" s="14" t="s">
+    </row>
+    <row r="73" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A73" s="2" t="s">
         <v>355</v>
       </c>
-      <c r="E67" s="3" t="s">
+      <c r="B73" s="14" t="s">
         <v>356</v>
       </c>
-      <c r="F67" s="36" t="s">
+      <c r="C73" s="14" t="s">
         <v>357</v>
       </c>
-      <c r="G67" s="8" t="s">
+      <c r="D73" s="14" t="s">
         <v>358</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A68" s="11" t="s">
-        <v>359</v>
-      </c>
-      <c r="B68" s="14" t="s">
-        <v>360</v>
-      </c>
-      <c r="C68" s="14" t="s">
-        <v>360</v>
-      </c>
-      <c r="D68" s="14" t="s">
-        <v>330</v>
-      </c>
-      <c r="E68" s="3" t="s">
-        <v>361</v>
-      </c>
-      <c r="F68" s="36" t="s">
-        <v>332</v>
-      </c>
-      <c r="G68" s="8" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A69" s="11" t="s">
-        <v>362</v>
-      </c>
-      <c r="B69" s="14" t="s">
-        <v>363</v>
-      </c>
-      <c r="C69" s="14" t="s">
-        <v>364</v>
-      </c>
-      <c r="D69" s="14" t="s">
-        <v>365</v>
-      </c>
-      <c r="E69" s="3" t="s">
-        <v>366</v>
-      </c>
-      <c r="F69" s="36" t="s">
-        <v>367</v>
-      </c>
-      <c r="G69" s="8" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A71" s="29" t="s">
-        <v>368</v>
-      </c>
-      <c r="B71" s="27"/>
-      <c r="C71" s="27"/>
-      <c r="D71" s="27"/>
-      <c r="E71" s="27"/>
-      <c r="F71" s="27"/>
-      <c r="G71" s="27"/>
-    </row>
-    <row r="72" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A72" s="1" t="s">
-        <v>369</v>
-      </c>
-      <c r="B72" s="1" t="s">
-        <v>370</v>
-      </c>
-      <c r="C72" s="1" t="s">
-        <v>371</v>
-      </c>
-      <c r="D72" s="1" t="s">
-        <v>372</v>
-      </c>
-      <c r="E72" s="1" t="s">
-        <v>373</v>
-      </c>
-      <c r="F72" s="34" t="s">
-        <v>374</v>
-      </c>
-      <c r="G72" s="1" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="73" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A73" s="2" t="s">
-        <v>376</v>
-      </c>
-      <c r="B73" s="14" t="s">
-        <v>377</v>
-      </c>
-      <c r="C73" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="D73" s="14" t="s">
-        <v>379</v>
       </c>
       <c r="E73" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="F73" s="37" t="s">
-        <v>380</v>
-      </c>
-      <c r="G73" s="3" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="74" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F73" s="30" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="2" t="s">
-        <v>382</v>
+        <v>360</v>
       </c>
       <c r="B74" s="14" t="s">
-        <v>383</v>
+        <v>361</v>
       </c>
       <c r="C74" s="14" t="s">
-        <v>384</v>
+        <v>362</v>
       </c>
       <c r="D74" s="14" t="s">
-        <v>385</v>
+        <v>363</v>
       </c>
       <c r="E74" s="9" t="s">
-        <v>386</v>
-      </c>
-      <c r="F74" s="37" t="s">
-        <v>380</v>
-      </c>
-      <c r="G74" s="3" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="75" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+        <v>364</v>
+      </c>
+      <c r="F74" s="30" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="2" t="s">
-        <v>388</v>
+        <v>365</v>
       </c>
       <c r="B75" s="14" t="s">
-        <v>389</v>
+        <v>366</v>
       </c>
       <c r="C75" s="14" t="s">
-        <v>390</v>
+        <v>367</v>
       </c>
       <c r="D75" s="14" t="s">
-        <v>391</v>
+        <v>368</v>
       </c>
       <c r="E75" s="9" t="s">
-        <v>392</v>
-      </c>
-      <c r="F75" s="37" t="s">
-        <v>380</v>
-      </c>
-      <c r="G75" s="3" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="77" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A77" s="29" t="s">
-        <v>394</v>
-      </c>
-      <c r="B77" s="27"/>
-      <c r="C77" s="27"/>
-      <c r="D77" s="27"/>
-      <c r="E77" s="27"/>
-      <c r="F77" s="27"/>
-      <c r="G77" s="27"/>
-    </row>
-    <row r="78" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.35">
+        <v>369</v>
+      </c>
+      <c r="F75" s="30" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A77" s="32" t="s">
+        <v>370</v>
+      </c>
+      <c r="B77" s="33"/>
+      <c r="C77" s="33"/>
+      <c r="D77" s="33"/>
+      <c r="E77" s="33"/>
+      <c r="F77" s="33"/>
+    </row>
+    <row r="78" spans="1:6" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
-        <v>395</v>
+        <v>371</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>396</v>
+        <v>372</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>397</v>
+        <v>373</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>398</v>
+        <v>374</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>399</v>
-      </c>
-      <c r="F78" s="34" t="s">
-        <v>400</v>
-      </c>
-      <c r="G78" s="1" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="79" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+        <v>375</v>
+      </c>
+      <c r="F78" s="27" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="3" t="s">
-        <v>402</v>
+        <v>377</v>
       </c>
       <c r="B79" s="14">
         <v>6</v>
@@ -5645,21 +5471,18 @@
         <v>60</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>403</v>
+        <v>378</v>
       </c>
       <c r="E79" s="14" t="s">
-        <v>404</v>
-      </c>
-      <c r="F79" s="37" t="s">
-        <v>405</v>
-      </c>
-      <c r="G79" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="80" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+        <v>379</v>
+      </c>
+      <c r="F79" s="30" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="3" t="s">
-        <v>407</v>
+        <v>381</v>
       </c>
       <c r="B80" s="14">
         <v>6</v>
@@ -5668,21 +5491,18 @@
         <v>60</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>403</v>
+        <v>378</v>
       </c>
       <c r="E80" s="14" t="s">
-        <v>408</v>
-      </c>
-      <c r="F80" s="37" t="s">
-        <v>409</v>
-      </c>
-      <c r="G80" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="81" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+        <v>382</v>
+      </c>
+      <c r="F80" s="30" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="3" t="s">
-        <v>410</v>
+        <v>384</v>
       </c>
       <c r="B81" s="14">
         <v>6</v>
@@ -5691,21 +5511,18 @@
         <v>60</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>403</v>
+        <v>378</v>
       </c>
       <c r="E81" s="14" t="s">
-        <v>411</v>
-      </c>
-      <c r="F81" s="37" t="s">
-        <v>412</v>
-      </c>
-      <c r="G81" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="82" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+        <v>385</v>
+      </c>
+      <c r="F81" s="30" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="3" t="s">
-        <v>413</v>
+        <v>387</v>
       </c>
       <c r="B82" s="14">
         <v>6</v>
@@ -5714,21 +5531,18 @@
         <v>60</v>
       </c>
       <c r="D82" s="4" t="s">
-        <v>403</v>
+        <v>378</v>
       </c>
       <c r="E82" s="14" t="s">
-        <v>414</v>
-      </c>
-      <c r="F82" s="37" t="s">
-        <v>415</v>
-      </c>
-      <c r="G82" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="83" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+        <v>388</v>
+      </c>
+      <c r="F82" s="30" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" s="3" t="s">
-        <v>416</v>
+        <v>390</v>
       </c>
       <c r="B83" s="14">
         <v>6</v>
@@ -5737,21 +5551,18 @@
         <v>60</v>
       </c>
       <c r="D83" s="4" t="s">
-        <v>403</v>
+        <v>378</v>
       </c>
       <c r="E83" s="14" t="s">
-        <v>417</v>
-      </c>
-      <c r="F83" s="37" t="s">
-        <v>418</v>
-      </c>
-      <c r="G83" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+        <v>391</v>
+      </c>
+      <c r="F83" s="30" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="3" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="B84" s="14">
         <v>6</v>
@@ -5760,21 +5571,18 @@
         <v>60</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>403</v>
+        <v>378</v>
       </c>
       <c r="E84" s="14" t="s">
-        <v>404</v>
-      </c>
-      <c r="F84" s="37" t="s">
-        <v>405</v>
-      </c>
-      <c r="G84" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="85" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+        <v>379</v>
+      </c>
+      <c r="F84" s="30" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="3" t="s">
-        <v>420</v>
+        <v>394</v>
       </c>
       <c r="B85" s="14">
         <v>6</v>
@@ -5783,21 +5591,18 @@
         <v>60</v>
       </c>
       <c r="D85" s="4" t="s">
-        <v>403</v>
+        <v>378</v>
       </c>
       <c r="E85" s="14" t="s">
-        <v>411</v>
-      </c>
-      <c r="F85" s="37" t="s">
-        <v>412</v>
-      </c>
-      <c r="G85" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+        <v>385</v>
+      </c>
+      <c r="F85" s="30" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86" s="3" t="s">
-        <v>421</v>
+        <v>395</v>
       </c>
       <c r="B86" s="14">
         <v>6</v>
@@ -5806,21 +5611,18 @@
         <v>60</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>403</v>
+        <v>378</v>
       </c>
       <c r="E86" s="14" t="s">
-        <v>404</v>
-      </c>
-      <c r="F86" s="37" t="s">
-        <v>405</v>
-      </c>
-      <c r="G86" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="87" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+        <v>379</v>
+      </c>
+      <c r="F86" s="30" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="3" t="s">
-        <v>422</v>
+        <v>396</v>
       </c>
       <c r="B87" s="14">
         <v>6</v>
@@ -5829,21 +5631,18 @@
         <v>60</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>403</v>
+        <v>378</v>
       </c>
       <c r="E87" s="14" t="s">
-        <v>417</v>
-      </c>
-      <c r="F87" s="37" t="s">
-        <v>418</v>
-      </c>
-      <c r="G87" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="88" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+        <v>391</v>
+      </c>
+      <c r="F87" s="30" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="3" t="s">
-        <v>423</v>
+        <v>397</v>
       </c>
       <c r="B88" s="14">
         <v>6</v>
@@ -5852,21 +5651,18 @@
         <v>60</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>403</v>
+        <v>378</v>
       </c>
       <c r="E88" s="14" t="s">
-        <v>404</v>
-      </c>
-      <c r="F88" s="37" t="s">
-        <v>405</v>
-      </c>
-      <c r="G88" s="8" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="89" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+        <v>379</v>
+      </c>
+      <c r="F88" s="30" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" s="20" t="s">
-        <v>424</v>
+        <v>398</v>
       </c>
       <c r="B89" s="24">
         <v>60</v>
@@ -5875,27 +5671,24 @@
         <v>600</v>
       </c>
       <c r="D89" s="5" t="s">
-        <v>403</v>
+        <v>378</v>
       </c>
       <c r="E89" s="24" t="s">
-        <v>425</v>
-      </c>
-      <c r="F89" s="38" t="s">
-        <v>426</v>
-      </c>
-      <c r="G89" s="8" t="s">
-        <v>406</v>
+        <v>399</v>
+      </c>
+      <c r="F89" s="31" t="s">
+        <v>400</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A61:G61"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A77:G77"/>
-    <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A71:G71"/>
-    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="A61:F61"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A77:F77"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A71:F71"/>
+    <mergeCell ref="A37:F37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>

</xml_diff>